<commit_message>
fix: batch encoding with chcp 65001
</commit_message>
<xml_diff>
--- a/搜索词示例.xlsx
+++ b/搜索词示例.xlsx
@@ -1,40 +1,203 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\junie\openclaw\google_searcher\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AE5C10D-A273-4741-B391-32A977CBAF5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="39">
+  <si>
+    <t>搜索词</t>
+  </si>
+  <si>
+    <t>保留关键词</t>
+  </si>
+  <si>
+    <t>Ruizhe Chen</t>
+  </si>
+  <si>
+    <t>Chunjiang Ge</t>
+  </si>
+  <si>
+    <t>Qidong Huang</t>
+  </si>
+  <si>
+    <t>Jie Huang</t>
+  </si>
+  <si>
+    <t>Shutong Jiang</t>
+  </si>
+  <si>
+    <t>Mingsheng Li</t>
+  </si>
+  <si>
+    <t>Zicheng Lin</t>
+  </si>
+  <si>
+    <t>Jiawei Liu</t>
+  </si>
+  <si>
+    <t>Chenglong Liu</t>
+  </si>
+  <si>
+    <t>Yang Liu</t>
+  </si>
+  <si>
+    <t>Dunjie Lu</t>
+  </si>
+  <si>
+    <t>Ruilin Luo</t>
+  </si>
+  <si>
+    <t>Lingchen Meng</t>
+  </si>
+  <si>
+    <t>Yuchong Sun</t>
+  </si>
+  <si>
+    <t>Qiuyue Wang</t>
+  </si>
+  <si>
+    <t>Fei Zhang</t>
+  </si>
+  <si>
+    <t>Ke Zhu</t>
+  </si>
+  <si>
+    <t>alibaba</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>+</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Ruizhe Chen+alibaba</t>
+  </si>
+  <si>
+    <t>Chunjiang Ge+alibaba</t>
+  </si>
+  <si>
+    <t>Qidong Huang+alibaba</t>
+  </si>
+  <si>
+    <t>Jie Huang+alibaba</t>
+  </si>
+  <si>
+    <t>Shutong Jiang+alibaba</t>
+  </si>
+  <si>
+    <t>Mingsheng Li+alibaba</t>
+  </si>
+  <si>
+    <t>Zicheng Lin+alibaba</t>
+  </si>
+  <si>
+    <t>Jiawei Liu+alibaba</t>
+  </si>
+  <si>
+    <t>Chenglong Liu+alibaba</t>
+  </si>
+  <si>
+    <t>Yang Liu+alibaba</t>
+  </si>
+  <si>
+    <t>Dunjie Lu+alibaba</t>
+  </si>
+  <si>
+    <t>Ruilin Luo+alibaba</t>
+  </si>
+  <si>
+    <t>Lingchen Meng+alibaba</t>
+  </si>
+  <si>
+    <t>Yuchong Sun+alibaba</t>
+  </si>
+  <si>
+    <t>Qiuyue Wang+alibaba</t>
+  </si>
+  <si>
+    <t>Fei Zhang+alibaba</t>
+  </si>
+  <si>
+    <t>Ke Zhu+alibaba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">scholar,github,openreview </t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <name val="Calibri"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color theme="1"/>
-      <sz val="11"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,85 +205,44 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFDEE0E3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFDEE0E3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFDEE0E3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFDEE0E3"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -408,59 +530,383 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <cols>
+    <col min="1" max="1" width="21" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>搜索词</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>保留关键词</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Python tkinter Windows清理工具</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>github.com</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>通义千问 开源论文 2025</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>arxiv</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Apple Design GUI toolkit</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" t="str">
+        <f>C2&amp;E2&amp;D2</f>
+        <v>Ruizhe Chen+alibaba</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" t="str">
+        <f t="shared" ref="F3:F18" si="0">C3&amp;E3&amp;D3</f>
+        <v>Chunjiang Ge+alibaba</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" t="str">
+        <f t="shared" si="0"/>
+        <v>Qidong Huang+alibaba</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A5" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" t="str">
+        <f t="shared" si="0"/>
+        <v>Jie Huang+alibaba</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" t="str">
+        <f t="shared" si="0"/>
+        <v>Shutong Jiang+alibaba</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D7" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" t="str">
+        <f t="shared" si="0"/>
+        <v>Mingsheng Li+alibaba</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" t="s">
+        <v>20</v>
+      </c>
+      <c r="F8" t="str">
+        <f t="shared" si="0"/>
+        <v>Zicheng Lin+alibaba</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F9" t="str">
+        <f t="shared" si="0"/>
+        <v>Jiawei Liu+alibaba</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10" t="str">
+        <f t="shared" si="0"/>
+        <v>Chenglong Liu+alibaba</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" t="s">
+        <v>19</v>
+      </c>
+      <c r="E11" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" t="str">
+        <f t="shared" si="0"/>
+        <v>Yang Liu+alibaba</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12" t="str">
+        <f t="shared" si="0"/>
+        <v>Dunjie Lu+alibaba</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A13" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13" t="str">
+        <f t="shared" si="0"/>
+        <v>Ruilin Luo+alibaba</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A14" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B14" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" t="str">
+        <f t="shared" si="0"/>
+        <v>Lingchen Meng+alibaba</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A15" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E15" t="s">
+        <v>20</v>
+      </c>
+      <c r="F15" t="str">
+        <f t="shared" si="0"/>
+        <v>Yuchong Sun+alibaba</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A16" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" t="s">
+        <v>38</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D16" t="s">
+        <v>19</v>
+      </c>
+      <c r="E16" t="s">
+        <v>20</v>
+      </c>
+      <c r="F16" t="str">
+        <f t="shared" si="0"/>
+        <v>Qiuyue Wang+alibaba</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D17" t="s">
+        <v>19</v>
+      </c>
+      <c r="E17" t="s">
+        <v>20</v>
+      </c>
+      <c r="F17" t="str">
+        <f t="shared" si="0"/>
+        <v>Fei Zhang+alibaba</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.15">
+      <c r="A18" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18" t="s">
+        <v>20</v>
+      </c>
+      <c r="F18" t="str">
+        <f t="shared" si="0"/>
+        <v>Ke Zhu+alibaba</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>